<commit_message>
Add Accommodation column to Merged sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FjL7728Xv291EiVCsdbaW7
</commit_message>
<xml_diff>
--- a/guest_list_anniversary.xlsx
+++ b/guest_list_anniversary.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Sheet1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Merged'!$A$4:$F$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Merged'!$A$4:$G$163</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Nishtara'!$A$4:$C$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Darling'!$A$4:$D$90</definedName>
   </definedNames>
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="B19" s="18">
-        <f>COUNTIF(Merged!$F$5:$F$163,"Both")</f>
+        <f>COUNTIF(Merged!$G$5:$G$163,"Both")</f>
         <v/>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="B20" s="18">
-        <f>COUNTIF(Merged!$F$5:$F$163,"Nishtara only")</f>
+        <f>COUNTIF(Merged!$G$5:$G$163,"Nishtara only")</f>
         <v/>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="B21" s="18">
-        <f>COUNTIF(Merged!$F$5:$F$163,"Darling only")</f>
+        <f>COUNTIF(Merged!$G$5:$G$163,"Darling only")</f>
         <v/>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:K163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1120,10 +1120,11 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1135,7 +1136,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5">
-        <f>COUNTA(B5:B163)&amp;" unique guests  |  Nishtara: "&amp;COUNTIF(D5:D163,"Yes")&amp;"  |  Darling: "&amp;COUNTIF(E5:E163,"Yes")&amp;"  |  Both: "&amp;COUNTIF(F5:F163,"Both")</f>
+        <f>COUNTA(B5:B163)&amp;" unique guests  |  Nishtara: "&amp;COUNTIF(D5:D163,"Yes")&amp;"  |  Darling: "&amp;COUNTIF(E5:E163,"Yes")&amp;"  |  Both: "&amp;COUNTIF(G5:G163,"Both")&amp;"  |  Accommodation: "&amp;COUNTIF(F5:F163,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1167,20 +1168,25 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
           <t>Invited To</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>Guests</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Go to list</t>
         </is>
@@ -1210,21 +1216,26 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G5" s="8">
         <f>IF(AND(D5="Yes",E5="Yes"),"Both",IF(D5="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>AJ 332</t>
         </is>
       </c>
-      <c r="I5" s="18">
-        <f>COUNTIF($C$5:$C$163,H5)</f>
-        <v/>
-      </c>
-      <c r="J5" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H5,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J5" s="18">
+        <f>COUNTIF($C$5:$C$163,I5)</f>
+        <v/>
+      </c>
+      <c r="K5" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I5,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1252,21 +1263,26 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G6" s="8">
         <f>IF(AND(D6="Yes",E6="Yes"),"Both",IF(D6="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H6" s="17" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>BL - 12</t>
         </is>
       </c>
-      <c r="I6" s="18">
-        <f>COUNTIF($C$5:$C$163,H6)</f>
-        <v/>
-      </c>
-      <c r="J6" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H6,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J6" s="18">
+        <f>COUNTIF($C$5:$C$163,I6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I6,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1294,21 +1310,26 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G7" s="8">
         <f>IF(AND(D7="Yes",E7="Yes"),"Both",IF(D7="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H7" s="17" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>Bhuaji</t>
         </is>
       </c>
-      <c r="I7" s="18">
-        <f>COUNTIF($C$5:$C$163,H7)</f>
-        <v/>
-      </c>
-      <c r="J7" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H7,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J7" s="18">
+        <f>COUNTIF($C$5:$C$163,I7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I7,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1336,21 +1357,26 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G8" s="8">
         <f>IF(AND(D8="Yes",E8="Yes"),"Both",IF(D8="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>Chaibasa</t>
         </is>
       </c>
-      <c r="I8" s="18">
-        <f>COUNTIF($C$5:$C$163,H8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H8,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J8" s="18">
+        <f>COUNTIF($C$5:$C$163,I8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I8,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1378,21 +1404,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="8">
         <f>IF(AND(D9="Yes",E9="Yes"),"Both",IF(D9="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>Deep Friend</t>
         </is>
       </c>
-      <c r="I9" s="18">
-        <f>COUNTIF($C$5:$C$163,H9)</f>
-        <v/>
-      </c>
-      <c r="J9" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H9,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J9" s="18">
+        <f>COUNTIF($C$5:$C$163,I9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I9,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1420,21 +1451,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" s="8">
         <f>IF(AND(D10="Yes",E10="Yes"),"Both",IF(D10="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>Maggi Friend</t>
         </is>
       </c>
-      <c r="I10" s="18">
-        <f>COUNTIF($C$5:$C$163,H10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H10,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J10" s="18">
+        <f>COUNTIF($C$5:$C$163,I10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I10,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1462,21 +1498,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="8">
         <f>IF(AND(D11="Yes",E11="Yes"),"Both",IF(D11="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>Manjari Friend</t>
         </is>
       </c>
-      <c r="I11" s="18">
-        <f>COUNTIF($C$5:$C$163,H11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H11,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J11" s="18">
+        <f>COUNTIF($C$5:$C$163,I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I11,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1504,21 +1545,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G12" s="8">
         <f>IF(AND(D12="Yes",E12="Yes"),"Both",IF(D12="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="I12" s="17" t="inlineStr">
         <is>
           <t>Nanibari</t>
         </is>
       </c>
-      <c r="I12" s="18">
-        <f>COUNTIF($C$5:$C$163,H12)</f>
-        <v/>
-      </c>
-      <c r="J12" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H12,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J12" s="18">
+        <f>COUNTIF($C$5:$C$163,I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I12,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1546,21 +1592,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G13" s="8">
         <f>IF(AND(D13="Yes",E13="Yes"),"Both",IF(D13="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="I13" s="17" t="inlineStr">
         <is>
           <t>Neighbour</t>
         </is>
       </c>
-      <c r="I13" s="18">
-        <f>COUNTIF($C$5:$C$163,H13)</f>
-        <v/>
-      </c>
-      <c r="J13" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H13,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J13" s="18">
+        <f>COUNTIF($C$5:$C$163,I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I13,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1588,21 +1639,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G14" s="8">
         <f>IF(AND(D14="Yes",E14="Yes"),"Both",IF(D14="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H14" s="17" t="inlineStr">
+      <c r="I14" s="17" t="inlineStr">
         <is>
           <t>Purulia</t>
         </is>
       </c>
-      <c r="I14" s="18">
-        <f>COUNTIF($C$5:$C$163,H14)</f>
-        <v/>
-      </c>
-      <c r="J14" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H14,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J14" s="18">
+        <f>COUNTIF($C$5:$C$163,I14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I14,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1630,21 +1686,26 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G15" s="8">
         <f>IF(AND(D15="Yes",E15="Yes"),"Both",IF(D15="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H15" s="17" t="inlineStr">
+      <c r="I15" s="17" t="inlineStr">
         <is>
           <t>Vinay Friend</t>
         </is>
       </c>
-      <c r="I15" s="18">
-        <f>COUNTIF($C$5:$C$163,H15)</f>
-        <v/>
-      </c>
-      <c r="J15" s="22">
-        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(H15,$C$1:$C$163,0),"View list ►")</f>
+      <c r="J15" s="18">
+        <f>COUNTIF($C$5:$C$163,I15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="22">
+        <f>HYPERLINK("#'Merged'!A"&amp;MATCH(I15,$C$1:$C$163,0),"View list ►")</f>
         <v/>
       </c>
     </row>
@@ -1672,20 +1733,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" s="8">
         <f>IF(AND(D16="Yes",E16="Yes"),"Both",IF(D16="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
-      <c r="H16" s="24" t="inlineStr">
+      <c r="I16" s="24" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="I16" s="14">
-        <f>SUM(I5:I15)</f>
-        <v/>
-      </c>
-      <c r="J16" s="15">
+      <c r="J16" s="14">
+        <f>SUM(J5:J15)</f>
+        <v/>
+      </c>
+      <c r="K16" s="15">
         <f>HYPERLINK("#'Summary'!A1","◄ Back to Summary")</f>
         <v/>
       </c>
@@ -1714,7 +1780,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="8">
         <f>IF(AND(D17="Yes",E17="Yes"),"Both",IF(D17="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -1743,7 +1814,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G18" s="8">
         <f>IF(AND(D18="Yes",E18="Yes"),"Both",IF(D18="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -1772,7 +1848,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" s="8">
         <f>IF(AND(D19="Yes",E19="Yes"),"Both",IF(D19="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -1801,7 +1882,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F20" s="8">
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G20" s="8">
         <f>IF(AND(D20="Yes",E20="Yes"),"Both",IF(D20="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -1830,7 +1916,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F21" s="8">
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="8">
         <f>IF(AND(D21="Yes",E21="Yes"),"Both",IF(D21="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -1859,7 +1950,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F22" s="8">
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" s="8">
         <f>IF(AND(D22="Yes",E22="Yes"),"Both",IF(D22="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -1888,7 +1984,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F23" s="8">
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G23" s="8">
         <f>IF(AND(D23="Yes",E23="Yes"),"Both",IF(D23="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -1917,7 +2018,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F24" s="8">
+      <c r="F24" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G24" s="8">
         <f>IF(AND(D24="Yes",E24="Yes"),"Both",IF(D24="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -1946,7 +2052,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G25" s="8">
         <f>IF(AND(D25="Yes",E25="Yes"),"Both",IF(D25="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -1975,7 +2086,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F26" s="8">
+      <c r="F26" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G26" s="8">
         <f>IF(AND(D26="Yes",E26="Yes"),"Both",IF(D26="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2004,7 +2120,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G27" s="8">
         <f>IF(AND(D27="Yes",E27="Yes"),"Both",IF(D27="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2033,7 +2154,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" s="8">
         <f>IF(AND(D28="Yes",E28="Yes"),"Both",IF(D28="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2062,7 +2188,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" s="8">
         <f>IF(AND(D29="Yes",E29="Yes"),"Both",IF(D29="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2091,7 +2222,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F30" s="8">
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G30" s="8">
         <f>IF(AND(D30="Yes",E30="Yes"),"Both",IF(D30="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2120,7 +2256,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F31" s="8">
+      <c r="F31" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G31" s="8">
         <f>IF(AND(D31="Yes",E31="Yes"),"Both",IF(D31="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2149,7 +2290,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F32" s="8">
+      <c r="F32" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G32" s="8">
         <f>IF(AND(D32="Yes",E32="Yes"),"Both",IF(D32="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2178,7 +2324,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F33" s="8">
+      <c r="F33" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G33" s="8">
         <f>IF(AND(D33="Yes",E33="Yes"),"Both",IF(D33="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2207,7 +2358,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F34" s="8">
+      <c r="F34" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G34" s="8">
         <f>IF(AND(D34="Yes",E34="Yes"),"Both",IF(D34="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2236,7 +2392,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F35" s="8">
+      <c r="F35" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" s="8">
         <f>IF(AND(D35="Yes",E35="Yes"),"Both",IF(D35="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2265,7 +2426,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F36" s="8">
+      <c r="F36" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G36" s="8">
         <f>IF(AND(D36="Yes",E36="Yes"),"Both",IF(D36="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2294,7 +2460,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F37" s="8">
+      <c r="F37" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G37" s="8">
         <f>IF(AND(D37="Yes",E37="Yes"),"Both",IF(D37="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2323,7 +2494,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F38" s="8">
+      <c r="F38" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G38" s="8">
         <f>IF(AND(D38="Yes",E38="Yes"),"Both",IF(D38="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2352,7 +2528,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F39" s="8">
+      <c r="F39" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G39" s="8">
         <f>IF(AND(D39="Yes",E39="Yes"),"Both",IF(D39="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2381,7 +2562,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F40" s="8">
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" s="8">
         <f>IF(AND(D40="Yes",E40="Yes"),"Both",IF(D40="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2410,7 +2596,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F41" s="8">
+      <c r="F41" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G41" s="8">
         <f>IF(AND(D41="Yes",E41="Yes"),"Both",IF(D41="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2439,7 +2630,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F42" s="8">
+      <c r="F42" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G42" s="8">
         <f>IF(AND(D42="Yes",E42="Yes"),"Both",IF(D42="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2468,7 +2664,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F43" s="8">
+      <c r="F43" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G43" s="8">
         <f>IF(AND(D43="Yes",E43="Yes"),"Both",IF(D43="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2497,7 +2698,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F44" s="8">
+      <c r="F44" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G44" s="8">
         <f>IF(AND(D44="Yes",E44="Yes"),"Both",IF(D44="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2526,7 +2732,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F45" s="8">
+      <c r="F45" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G45" s="8">
         <f>IF(AND(D45="Yes",E45="Yes"),"Both",IF(D45="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2555,7 +2766,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F46" s="8">
+      <c r="F46" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G46" s="8">
         <f>IF(AND(D46="Yes",E46="Yes"),"Both",IF(D46="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2584,7 +2800,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F47" s="8">
+      <c r="F47" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G47" s="8">
         <f>IF(AND(D47="Yes",E47="Yes"),"Both",IF(D47="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2613,7 +2834,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F48" s="8">
+      <c r="F48" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G48" s="8">
         <f>IF(AND(D48="Yes",E48="Yes"),"Both",IF(D48="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2642,7 +2868,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F49" s="8">
+      <c r="F49" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G49" s="8">
         <f>IF(AND(D49="Yes",E49="Yes"),"Both",IF(D49="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2671,7 +2902,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F50" s="8">
+      <c r="F50" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G50" s="8">
         <f>IF(AND(D50="Yes",E50="Yes"),"Both",IF(D50="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2700,7 +2936,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F51" s="8">
+      <c r="F51" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G51" s="8">
         <f>IF(AND(D51="Yes",E51="Yes"),"Both",IF(D51="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2729,7 +2970,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F52" s="8">
+      <c r="F52" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G52" s="8">
         <f>IF(AND(D52="Yes",E52="Yes"),"Both",IF(D52="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2758,7 +3004,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F53" s="8">
+      <c r="F53" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G53" s="8">
         <f>IF(AND(D53="Yes",E53="Yes"),"Both",IF(D53="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2787,7 +3038,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F54" s="8">
+      <c r="F54" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G54" s="8">
         <f>IF(AND(D54="Yes",E54="Yes"),"Both",IF(D54="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2816,7 +3072,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F55" s="8">
+      <c r="F55" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G55" s="8">
         <f>IF(AND(D55="Yes",E55="Yes"),"Both",IF(D55="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2845,7 +3106,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F56" s="8">
+      <c r="F56" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G56" s="8">
         <f>IF(AND(D56="Yes",E56="Yes"),"Both",IF(D56="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2874,7 +3140,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F57" s="8">
+      <c r="F57" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G57" s="8">
         <f>IF(AND(D57="Yes",E57="Yes"),"Both",IF(D57="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2903,7 +3174,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F58" s="8">
+      <c r="F58" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G58" s="8">
         <f>IF(AND(D58="Yes",E58="Yes"),"Both",IF(D58="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2932,7 +3208,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F59" s="8">
+      <c r="F59" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G59" s="8">
         <f>IF(AND(D59="Yes",E59="Yes"),"Both",IF(D59="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2961,7 +3242,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F60" s="8">
+      <c r="F60" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G60" s="8">
         <f>IF(AND(D60="Yes",E60="Yes"),"Both",IF(D60="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -2990,7 +3276,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F61" s="8">
+      <c r="F61" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G61" s="8">
         <f>IF(AND(D61="Yes",E61="Yes"),"Both",IF(D61="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3019,7 +3310,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F62" s="8">
+      <c r="F62" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G62" s="8">
         <f>IF(AND(D62="Yes",E62="Yes"),"Both",IF(D62="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3048,7 +3344,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F63" s="8">
+      <c r="F63" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G63" s="8">
         <f>IF(AND(D63="Yes",E63="Yes"),"Both",IF(D63="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3077,7 +3378,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F64" s="8">
+      <c r="F64" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G64" s="8">
         <f>IF(AND(D64="Yes",E64="Yes"),"Both",IF(D64="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3106,7 +3412,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F65" s="8">
+      <c r="F65" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G65" s="8">
         <f>IF(AND(D65="Yes",E65="Yes"),"Both",IF(D65="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3135,7 +3446,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F66" s="8">
+      <c r="F66" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G66" s="8">
         <f>IF(AND(D66="Yes",E66="Yes"),"Both",IF(D66="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3164,7 +3480,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F67" s="8">
+      <c r="F67" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G67" s="8">
         <f>IF(AND(D67="Yes",E67="Yes"),"Both",IF(D67="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3193,7 +3514,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F68" s="8">
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G68" s="8">
         <f>IF(AND(D68="Yes",E68="Yes"),"Both",IF(D68="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3222,7 +3548,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F69" s="8">
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G69" s="8">
         <f>IF(AND(D69="Yes",E69="Yes"),"Both",IF(D69="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3251,7 +3582,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F70" s="8">
+      <c r="F70" s="11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G70" s="8">
         <f>IF(AND(D70="Yes",E70="Yes"),"Both",IF(D70="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3280,7 +3616,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F71" s="8">
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G71" s="8">
         <f>IF(AND(D71="Yes",E71="Yes"),"Both",IF(D71="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3309,7 +3650,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F72" s="8">
+      <c r="F72" s="11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G72" s="8">
         <f>IF(AND(D72="Yes",E72="Yes"),"Both",IF(D72="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3338,7 +3684,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F73" s="8">
+      <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G73" s="8">
         <f>IF(AND(D73="Yes",E73="Yes"),"Both",IF(D73="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3367,7 +3718,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F74" s="8">
+      <c r="F74" s="11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G74" s="8">
         <f>IF(AND(D74="Yes",E74="Yes"),"Both",IF(D74="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3396,7 +3752,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F75" s="8">
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G75" s="8">
         <f>IF(AND(D75="Yes",E75="Yes"),"Both",IF(D75="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3425,7 +3786,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F76" s="8">
+      <c r="F76" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G76" s="8">
         <f>IF(AND(D76="Yes",E76="Yes"),"Both",IF(D76="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3454,7 +3820,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F77" s="8">
+      <c r="F77" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G77" s="8">
         <f>IF(AND(D77="Yes",E77="Yes"),"Both",IF(D77="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3483,7 +3854,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F78" s="8">
+      <c r="F78" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G78" s="8">
         <f>IF(AND(D78="Yes",E78="Yes"),"Both",IF(D78="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3512,7 +3888,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F79" s="8">
+      <c r="F79" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G79" s="8">
         <f>IF(AND(D79="Yes",E79="Yes"),"Both",IF(D79="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3541,7 +3922,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F80" s="8">
+      <c r="F80" s="11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G80" s="8">
         <f>IF(AND(D80="Yes",E80="Yes"),"Both",IF(D80="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3570,7 +3956,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F81" s="8">
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G81" s="8">
         <f>IF(AND(D81="Yes",E81="Yes"),"Both",IF(D81="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3599,7 +3990,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F82" s="8">
+      <c r="F82" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G82" s="8">
         <f>IF(AND(D82="Yes",E82="Yes"),"Both",IF(D82="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3628,7 +4024,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F83" s="8">
+      <c r="F83" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G83" s="8">
         <f>IF(AND(D83="Yes",E83="Yes"),"Both",IF(D83="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3657,7 +4058,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F84" s="8">
+      <c r="F84" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G84" s="8">
         <f>IF(AND(D84="Yes",E84="Yes"),"Both",IF(D84="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3686,7 +4092,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F85" s="8">
+      <c r="F85" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G85" s="8">
         <f>IF(AND(D85="Yes",E85="Yes"),"Both",IF(D85="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3715,7 +4126,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F86" s="8">
+      <c r="F86" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G86" s="8">
         <f>IF(AND(D86="Yes",E86="Yes"),"Both",IF(D86="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3744,7 +4160,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F87" s="8">
+      <c r="F87" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G87" s="8">
         <f>IF(AND(D87="Yes",E87="Yes"),"Both",IF(D87="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3773,7 +4194,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F88" s="8">
+      <c r="F88" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G88" s="8">
         <f>IF(AND(D88="Yes",E88="Yes"),"Both",IF(D88="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3802,7 +4228,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F89" s="8">
+      <c r="F89" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G89" s="8">
         <f>IF(AND(D89="Yes",E89="Yes"),"Both",IF(D89="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3831,7 +4262,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F90" s="8">
+      <c r="F90" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G90" s="8">
         <f>IF(AND(D90="Yes",E90="Yes"),"Both",IF(D90="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3860,7 +4296,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F91" s="8">
+      <c r="F91" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G91" s="8">
         <f>IF(AND(D91="Yes",E91="Yes"),"Both",IF(D91="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3889,7 +4330,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F92" s="8">
+      <c r="F92" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G92" s="8">
         <f>IF(AND(D92="Yes",E92="Yes"),"Both",IF(D92="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3918,7 +4364,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F93" s="8">
+      <c r="F93" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G93" s="8">
         <f>IF(AND(D93="Yes",E93="Yes"),"Both",IF(D93="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3947,7 +4398,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F94" s="8">
+      <c r="F94" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G94" s="8">
         <f>IF(AND(D94="Yes",E94="Yes"),"Both",IF(D94="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -3976,7 +4432,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F95" s="8">
+      <c r="F95" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G95" s="8">
         <f>IF(AND(D95="Yes",E95="Yes"),"Both",IF(D95="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4005,7 +4466,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F96" s="8">
+      <c r="F96" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G96" s="8">
         <f>IF(AND(D96="Yes",E96="Yes"),"Both",IF(D96="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4034,7 +4500,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F97" s="8">
+      <c r="F97" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G97" s="8">
         <f>IF(AND(D97="Yes",E97="Yes"),"Both",IF(D97="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4063,7 +4534,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F98" s="8">
+      <c r="F98" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G98" s="8">
         <f>IF(AND(D98="Yes",E98="Yes"),"Both",IF(D98="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4092,7 +4568,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F99" s="8">
+      <c r="F99" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G99" s="8">
         <f>IF(AND(D99="Yes",E99="Yes"),"Both",IF(D99="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4121,7 +4602,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F100" s="8">
+      <c r="F100" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G100" s="8">
         <f>IF(AND(D100="Yes",E100="Yes"),"Both",IF(D100="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4150,7 +4636,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F101" s="8">
+      <c r="F101" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G101" s="8">
         <f>IF(AND(D101="Yes",E101="Yes"),"Both",IF(D101="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4179,7 +4670,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F102" s="8">
+      <c r="F102" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G102" s="8">
         <f>IF(AND(D102="Yes",E102="Yes"),"Both",IF(D102="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4208,7 +4704,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F103" s="8">
+      <c r="F103" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G103" s="8">
         <f>IF(AND(D103="Yes",E103="Yes"),"Both",IF(D103="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4237,7 +4738,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F104" s="8">
+      <c r="F104" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G104" s="8">
         <f>IF(AND(D104="Yes",E104="Yes"),"Both",IF(D104="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4266,7 +4772,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F105" s="8">
+      <c r="F105" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G105" s="8">
         <f>IF(AND(D105="Yes",E105="Yes"),"Both",IF(D105="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4295,7 +4806,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F106" s="8">
+      <c r="F106" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G106" s="8">
         <f>IF(AND(D106="Yes",E106="Yes"),"Both",IF(D106="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4324,7 +4840,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F107" s="8">
+      <c r="F107" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G107" s="8">
         <f>IF(AND(D107="Yes",E107="Yes"),"Both",IF(D107="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4353,7 +4874,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F108" s="8">
+      <c r="F108" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G108" s="8">
         <f>IF(AND(D108="Yes",E108="Yes"),"Both",IF(D108="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4382,7 +4908,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F109" s="8">
+      <c r="F109" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G109" s="8">
         <f>IF(AND(D109="Yes",E109="Yes"),"Both",IF(D109="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4411,7 +4942,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F110" s="8">
+      <c r="F110" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G110" s="8">
         <f>IF(AND(D110="Yes",E110="Yes"),"Both",IF(D110="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4440,7 +4976,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F111" s="8">
+      <c r="F111" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G111" s="8">
         <f>IF(AND(D111="Yes",E111="Yes"),"Both",IF(D111="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4469,7 +5010,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F112" s="8">
+      <c r="F112" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G112" s="8">
         <f>IF(AND(D112="Yes",E112="Yes"),"Both",IF(D112="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4498,7 +5044,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F113" s="8">
+      <c r="F113" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G113" s="8">
         <f>IF(AND(D113="Yes",E113="Yes"),"Both",IF(D113="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4527,7 +5078,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F114" s="8">
+      <c r="F114" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G114" s="8">
         <f>IF(AND(D114="Yes",E114="Yes"),"Both",IF(D114="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4556,7 +5112,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F115" s="8">
+      <c r="F115" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G115" s="8">
         <f>IF(AND(D115="Yes",E115="Yes"),"Both",IF(D115="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4585,7 +5146,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F116" s="8">
+      <c r="F116" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G116" s="8">
         <f>IF(AND(D116="Yes",E116="Yes"),"Both",IF(D116="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4614,7 +5180,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F117" s="8">
+      <c r="F117" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G117" s="8">
         <f>IF(AND(D117="Yes",E117="Yes"),"Both",IF(D117="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4643,7 +5214,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F118" s="8">
+      <c r="F118" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G118" s="8">
         <f>IF(AND(D118="Yes",E118="Yes"),"Both",IF(D118="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4672,7 +5248,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F119" s="8">
+      <c r="F119" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G119" s="8">
         <f>IF(AND(D119="Yes",E119="Yes"),"Both",IF(D119="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4701,7 +5282,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F120" s="8">
+      <c r="F120" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G120" s="8">
         <f>IF(AND(D120="Yes",E120="Yes"),"Both",IF(D120="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4730,7 +5316,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F121" s="8">
+      <c r="F121" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G121" s="8">
         <f>IF(AND(D121="Yes",E121="Yes"),"Both",IF(D121="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4759,7 +5350,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F122" s="8">
+      <c r="F122" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G122" s="8">
         <f>IF(AND(D122="Yes",E122="Yes"),"Both",IF(D122="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4788,7 +5384,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F123" s="8">
+      <c r="F123" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G123" s="8">
         <f>IF(AND(D123="Yes",E123="Yes"),"Both",IF(D123="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4817,7 +5418,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F124" s="8">
+      <c r="F124" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G124" s="8">
         <f>IF(AND(D124="Yes",E124="Yes"),"Both",IF(D124="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4846,7 +5452,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F125" s="8">
+      <c r="F125" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G125" s="8">
         <f>IF(AND(D125="Yes",E125="Yes"),"Both",IF(D125="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4875,7 +5486,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F126" s="8">
+      <c r="F126" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G126" s="8">
         <f>IF(AND(D126="Yes",E126="Yes"),"Both",IF(D126="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4904,7 +5520,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F127" s="8">
+      <c r="F127" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G127" s="8">
         <f>IF(AND(D127="Yes",E127="Yes"),"Both",IF(D127="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4933,7 +5554,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F128" s="8">
+      <c r="F128" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G128" s="8">
         <f>IF(AND(D128="Yes",E128="Yes"),"Both",IF(D128="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4962,7 +5588,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F129" s="8">
+      <c r="F129" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G129" s="8">
         <f>IF(AND(D129="Yes",E129="Yes"),"Both",IF(D129="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -4991,7 +5622,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F130" s="8">
+      <c r="F130" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G130" s="8">
         <f>IF(AND(D130="Yes",E130="Yes"),"Both",IF(D130="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5020,7 +5656,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F131" s="8">
+      <c r="F131" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G131" s="8">
         <f>IF(AND(D131="Yes",E131="Yes"),"Both",IF(D131="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5049,7 +5690,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F132" s="8">
+      <c r="F132" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G132" s="8">
         <f>IF(AND(D132="Yes",E132="Yes"),"Both",IF(D132="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5078,7 +5724,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F133" s="8">
+      <c r="F133" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G133" s="8">
         <f>IF(AND(D133="Yes",E133="Yes"),"Both",IF(D133="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5107,7 +5758,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F134" s="8">
+      <c r="F134" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G134" s="8">
         <f>IF(AND(D134="Yes",E134="Yes"),"Both",IF(D134="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5136,7 +5792,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F135" s="8">
+      <c r="F135" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G135" s="8">
         <f>IF(AND(D135="Yes",E135="Yes"),"Both",IF(D135="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5165,7 +5826,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F136" s="8">
+      <c r="F136" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G136" s="8">
         <f>IF(AND(D136="Yes",E136="Yes"),"Both",IF(D136="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5194,7 +5860,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F137" s="8">
+      <c r="F137" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G137" s="8">
         <f>IF(AND(D137="Yes",E137="Yes"),"Both",IF(D137="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5223,7 +5894,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F138" s="8">
+      <c r="F138" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G138" s="8">
         <f>IF(AND(D138="Yes",E138="Yes"),"Both",IF(D138="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5252,7 +5928,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F139" s="8">
+      <c r="F139" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G139" s="8">
         <f>IF(AND(D139="Yes",E139="Yes"),"Both",IF(D139="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5281,7 +5962,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F140" s="8">
+      <c r="F140" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G140" s="8">
         <f>IF(AND(D140="Yes",E140="Yes"),"Both",IF(D140="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5310,7 +5996,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F141" s="8">
+      <c r="F141" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G141" s="8">
         <f>IF(AND(D141="Yes",E141="Yes"),"Both",IF(D141="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5339,7 +6030,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F142" s="8">
+      <c r="F142" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G142" s="8">
         <f>IF(AND(D142="Yes",E142="Yes"),"Both",IF(D142="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5368,7 +6064,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F143" s="8">
+      <c r="F143" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G143" s="8">
         <f>IF(AND(D143="Yes",E143="Yes"),"Both",IF(D143="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5397,7 +6098,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F144" s="8">
+      <c r="F144" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G144" s="8">
         <f>IF(AND(D144="Yes",E144="Yes"),"Both",IF(D144="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5426,7 +6132,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F145" s="8">
+      <c r="F145" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G145" s="8">
         <f>IF(AND(D145="Yes",E145="Yes"),"Both",IF(D145="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5455,7 +6166,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F146" s="8">
+      <c r="F146" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G146" s="8">
         <f>IF(AND(D146="Yes",E146="Yes"),"Both",IF(D146="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5484,7 +6200,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F147" s="8">
+      <c r="F147" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G147" s="8">
         <f>IF(AND(D147="Yes",E147="Yes"),"Both",IF(D147="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5513,7 +6234,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F148" s="8">
+      <c r="F148" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G148" s="8">
         <f>IF(AND(D148="Yes",E148="Yes"),"Both",IF(D148="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5542,7 +6268,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F149" s="8">
+      <c r="F149" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G149" s="8">
         <f>IF(AND(D149="Yes",E149="Yes"),"Both",IF(D149="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5571,7 +6302,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F150" s="8">
+      <c r="F150" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G150" s="8">
         <f>IF(AND(D150="Yes",E150="Yes"),"Both",IF(D150="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5600,7 +6336,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F151" s="8">
+      <c r="F151" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G151" s="8">
         <f>IF(AND(D151="Yes",E151="Yes"),"Both",IF(D151="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5629,7 +6370,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F152" s="8">
+      <c r="F152" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G152" s="8">
         <f>IF(AND(D152="Yes",E152="Yes"),"Both",IF(D152="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5658,7 +6404,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F153" s="8">
+      <c r="F153" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G153" s="8">
         <f>IF(AND(D153="Yes",E153="Yes"),"Both",IF(D153="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5687,7 +6438,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F154" s="8">
+      <c r="F154" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G154" s="8">
         <f>IF(AND(D154="Yes",E154="Yes"),"Both",IF(D154="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5716,7 +6472,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F155" s="8">
+      <c r="F155" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G155" s="8">
         <f>IF(AND(D155="Yes",E155="Yes"),"Both",IF(D155="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5745,7 +6506,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F156" s="8">
+      <c r="F156" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G156" s="8">
         <f>IF(AND(D156="Yes",E156="Yes"),"Both",IF(D156="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5774,7 +6540,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F157" s="8">
+      <c r="F157" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G157" s="8">
         <f>IF(AND(D157="Yes",E157="Yes"),"Both",IF(D157="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5803,7 +6574,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F158" s="8">
+      <c r="F158" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G158" s="8">
         <f>IF(AND(D158="Yes",E158="Yes"),"Both",IF(D158="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5832,7 +6608,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F159" s="8">
+      <c r="F159" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G159" s="8">
         <f>IF(AND(D159="Yes",E159="Yes"),"Both",IF(D159="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5861,7 +6642,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F160" s="8">
+      <c r="F160" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G160" s="8">
         <f>IF(AND(D160="Yes",E160="Yes"),"Both",IF(D160="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5890,7 +6676,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F161" s="8">
+      <c r="F161" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G161" s="8">
         <f>IF(AND(D161="Yes",E161="Yes"),"Both",IF(D161="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5919,7 +6710,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F162" s="8">
+      <c r="F162" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G162" s="8">
         <f>IF(AND(D162="Yes",E162="Yes"),"Both",IF(D162="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
@@ -5948,13 +6744,18 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F163" s="8">
+      <c r="F163" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G163" s="8">
         <f>IF(AND(D163="Yes",E163="Yes"),"Both",IF(D163="Yes","Nishtara only","Darling only"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F163"/>
+  <autoFilter ref="A4:G163"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>